<commit_message>
Work in progress: wording sweep (left off the draft, deleted after it), agents still running
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012JjD5mhtvLxzAXoZHMZYE5
</commit_message>
<xml_diff>
--- a/downloads/assam.xlsx
+++ b/downloads/assam.xlsx
@@ -13105,7 +13105,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Kept out of the verification register. Carried forward to the draft unchanged. Removed or changed only on an order of a Foreigners Tribunal or a court</t>
+          <t>Kept out of the verification register. Carried forward to the draft unchanged. Deleted or changed only on an order of a Foreigners Tribunal or a court</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -13216,7 +13216,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Multiple entries, dead and permanently shifted electors removed through Form 7 before the draft</t>
+          <t>Multiple entries, dead and permanently shifted electors deleted through Form 7 before the draft</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">

</xml_diff>